<commit_message>
changes to forecast accuracy chart and technical guidance
</commit_message>
<xml_diff>
--- a/data/tech_guidance.xlsx
+++ b/data/tech_guidance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rmiller3\repos\la-school-places-scorecard-internal\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jbrett\repos\la-school-places-scorecards\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62591664-EEA0-428C-BFDE-3207C90A1360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12CB439D-05BA-4DB1-B6A5-55831A0081A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{9CCC1F63-2262-45DD-B4CA-7C937E5C8E7F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{9CCC1F63-2262-45DD-B4CA-7C937E5C8E7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Quantity" sheetId="2" r:id="rId1"/>
@@ -1361,6 +1361,39 @@
     </r>
   </si>
   <si>
+    <t>1. Each school has been matched with the Ofsted data as at  31 August 2025 (published November 2025). Graded judgements on four areas 'Quality of Education', 'Behaviour and Attitudes', 'Personal Development' and 'Leadership and Management' are used and where the inspection took place before 1 September 2023 the rating for 'Overall effectiveness: how good is the school is." is used for each judgement area.
+&lt;br&gt;2. There are four Ofsted categories: 'Outstanding', 'Good', 'Requires improvement' and 'Inadequate'.
+&lt;br&gt;3. The calculation counts the number of existing and new places that have been created in schools of each category. &lt;br&gt;4. Note that many schools will have been inspected some time before August 2025, and some will have been inspected since this date. &lt;br&gt;5. There are school places with no rating, as the school has yet to be inspected so do not have an Ofsted judgement.</t>
+  </si>
+  <si>
+    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2027/28 as provided in SCAP 2025.
+&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
+&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
+&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
+  </si>
+  <si>
+    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2026/27 as provided in SCAP 2024.
+&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
+&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
+&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
+  </si>
+  <si>
+    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2025/26 as provided in SCAP 2023.
+&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
+&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
+&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
+  </si>
+  <si>
+    <t>Total basic need funding 2011 to 2028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total amount of basic need capital funding allocated to each local authority to support them to create new mainstream primary and secondary places from 2011 to 2028. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. This refers to the amount of basic need capital funding that the Department for Education (DfE) has allocated to each local authority to create new places from the 2011-12 financial year to the 2027-28 financial year. Basic Need funding for the 2027-28 financial year is intended to support the creation of mainstream places for pupils aged 5 to 16 for the 2028/29 academic year. &lt;br&gt;2. The figure includes formula-based funding allocations and funding provided through the Targeted Basic Need Programme. Basic Need formula-based funding allocations cover the whole period and are not ring-fenced (although they can only be used for capital purposes).  Targeted Basic Need funding was provided between 2013 and 2015 and had to be spent by agreed deadlines and on specific projects. Both types of allocations are published here. &lt;br&gt;3. The figure only includes funding allocated to local authorities and does not include centrally-funded capital programmes such as the free schools programme. &lt;br&gt;4. The England total will not match the sum of allocations for all local authorities in the scorecard because the England total includes allocations to predecessor local authorities.
+</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">1. The cost data used in the scorecard is the 2018 Capital Spend data as used in the scorecards since 2018. For the 2025 Scorecard, this data has been adjusted for inflation (rebased to 1st Quarter 2026 prices). National averages adjusted for 2023 regional location factors are shown. You can use this data to establish developer contributions per school place, by adjusting for further inflation if needed (see examples below).
 &lt;br&gt;2. Projects which do not create additional mainstream places or where the project's additional place funding is zero are removed.
@@ -1465,7 +1498,7 @@
 &lt;br&gt;6. The average cost includes costs associated with maintenance and building condition or enhancement works.
 &lt;br&gt;7. The measure does not include places in special schools or units attached to mainstream schools, or new places which were funded through central programmes (including free schools). For projects within the 2018 Capital Spend dataset, a project which creates additional mainstream places and also creates SEN places or re-provides places, has been adjusted to apportion out those costs. For projects within the Capital Spend Survey, apportioning costs is not possible and therefore a project which creates additional mainstream places and also creates SEN places or re-provides places has been excluded.
 &lt;br&gt;8. All costs have been normalised to a common UK average price level using regional location factors published by BCIS, March 2023, 1 is the base weight.
-&lt;br&gt;9. All costs have been adjusted for inflation using the latest BCIS All-In Tender Price of Index (TPI), published March 2026.  Costs have been rebased from the start of construction (or time of place provision if construction start date unavailable) to 1st Quarter (Jan – Mar) 2026 prices using this index (Q1 2026 index value = 399).
+&lt;br&gt;9. All costs have been adjusted for inflation using the latest BCIS All-In Tender Price of Index (TPI), published March 2026.  Costs have been rebased from the start of construction (or time of place provision if construction start date unavailable) to 1st Quarter (Jan – Mar) 2026 prices using this index (Q1 2026 index value = 410).
 10. </t>
     </r>
     <r>
@@ -1485,42 +1518,9 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>.  If you have access to the BCIS indices via a subscription to BCIS Online (https://www.rics.org/uk/products/data-products/bcis-construction/bcis-online/) you can use the latest inflation index to re-base (weight to apply = latest index/399).  If not, you can apply a known change to the published cost (e.g. up or down x%).
+      <t>.  If you have access to the BCIS indices via a subscription to BCIS Online (https://www.rics.org/uk/products/data-products/bcis-construction/bcis-online/) you can use the latest inflation index to re-base (weight to apply = latest index/410).  If not, you can apply a known change to the published cost (e.g. up or down x%).
 11. Some additional but limited benchmark information for similar capital programme schemes carried out by the DfE is available in the National School Delivery Cost Benchmarking study: https://documents.hants.gov.uk/property-services/NationalSchoolDeliveryBenchmarkingreport.pdf</t>
     </r>
-  </si>
-  <si>
-    <t>1. Each school has been matched with the Ofsted data as at  31 August 2025 (published November 2025). Graded judgements on four areas 'Quality of Education', 'Behaviour and Attitudes', 'Personal Development' and 'Leadership and Management' are used and where the inspection took place before 1 September 2023 the rating for 'Overall effectiveness: how good is the school is." is used for each judgement area.
-&lt;br&gt;2. There are four Ofsted categories: 'Outstanding', 'Good', 'Requires improvement' and 'Inadequate'.
-&lt;br&gt;3. The calculation counts the number of existing and new places that have been created in schools of each category. &lt;br&gt;4. Note that many schools will have been inspected some time before August 2025, and some will have been inspected since this date. &lt;br&gt;5. There are school places with no rating, as the school has yet to be inspected so do not have an Ofsted judgement.</t>
-  </si>
-  <si>
-    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2027/28 as provided in SCAP 2025.
-&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
-&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
-&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
-  </si>
-  <si>
-    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2026/27 as provided in SCAP 2024.
-&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
-&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
-&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
-  </si>
-  <si>
-    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2025/26 as provided in SCAP 2023.
-&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
-&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
-&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
-  </si>
-  <si>
-    <t>Total basic need funding 2011 to 2028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total amount of basic need capital funding allocated to each local authority to support them to create new mainstream primary and secondary places from 2011 to 2028. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. This refers to the amount of basic need capital funding that the Department for Education (DfE) has allocated to each local authority to create new places from the 2011-12 financial year to the 2027-28 financial year. Basic Need funding for the 2027-28 financial year is intended to support the creation of mainstream places for pupils aged 5 to 16 for the 2028/29 academic year. &lt;br&gt;2. The figure includes formula-based funding allocations and funding provided through the Targeted Basic Need Programme. Basic Need formula-based funding allocations cover the whole period and are not ring-fenced (although they can only be used for capital purposes).  Targeted Basic Need funding was provided between 2013 and 2015 and had to be spent by agreed deadlines and on specific projects. Both types of allocations are published here. &lt;br&gt;3. The figure only includes funding allocated to local authorities and does not include centrally-funded capital programmes such as the free schools programme. &lt;br&gt;4. The England total will not match the sum of allocations for all local authorities in the scorecard because the England total includes allocations to predecessor local authorities.
-</t>
   </si>
 </sst>
 </file>
@@ -2031,15 +2031,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2058,16 +2064,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2386,16 +2386,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8372DA64-5E2C-41C1-8CF4-85BC1C2AFF86}">
   <dimension ref="A1:F44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.7265625" customWidth="1"/>
-    <col min="2" max="2" width="29.54296875" customWidth="1"/>
-    <col min="3" max="3" width="54.26953125" customWidth="1"/>
-    <col min="4" max="4" width="28.7265625" customWidth="1"/>
-    <col min="5" max="5" width="87.26953125" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.5703125" customWidth="1"/>
+    <col min="3" max="3" width="54.28515625" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" customWidth="1"/>
+    <col min="5" max="5" width="87.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -2415,11 +2415,11 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="87" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="52" t="s">
         <v>33</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -2428,32 +2428,32 @@
       <c r="D2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="62" t="s">
+      <c r="E2" s="54" t="s">
         <v>34</v>
       </c>
       <c r="F2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="87" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
-      <c r="B3" s="54"/>
+      <c r="B3" s="53"/>
       <c r="C3" s="4" t="s">
         <v>231</v>
       </c>
       <c r="D3" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="54"/>
+      <c r="E3" s="53"/>
       <c r="F3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="138" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="138" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="55" t="s">
         <v>94</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -2469,9 +2469,9 @@
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
-      <c r="B5" s="53"/>
+      <c r="B5" s="56"/>
       <c r="C5" s="4" t="s">
         <v>24</v>
       </c>
@@ -2485,9 +2485,9 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
-      <c r="B6" s="53"/>
+      <c r="B6" s="56"/>
       <c r="C6" s="11" t="s">
         <v>42</v>
       </c>
@@ -2501,9 +2501,9 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="6"/>
-      <c r="B7" s="53"/>
+      <c r="B7" s="56"/>
       <c r="C7" s="11" t="s">
         <v>43</v>
       </c>
@@ -2517,9 +2517,9 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
-      <c r="B8" s="54"/>
+      <c r="B8" s="53"/>
       <c r="C8" s="11" t="s">
         <v>229</v>
       </c>
@@ -2531,7 +2531,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>46</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="375" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="s">
         <v>47</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="189" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" ht="210.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>50</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
         <v>54</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
       <c r="B13" s="19"/>
       <c r="C13" s="9" t="s">
@@ -2623,7 +2623,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7"/>
       <c r="B14" s="24"/>
       <c r="C14" s="28" t="s">
@@ -2633,17 +2633,17 @@
         <v>59</v>
       </c>
       <c r="E14" s="28" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F14" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="61" t="s">
+      <c r="B15" s="52" t="s">
         <v>130</v>
       </c>
       <c r="C15" s="3" t="s">
@@ -2652,32 +2652,32 @@
       <c r="D15" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E15" s="62" t="s">
+      <c r="E15" s="54" t="s">
         <v>105</v>
       </c>
       <c r="F15" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
-      <c r="B16" s="54"/>
+      <c r="B16" s="53"/>
       <c r="C16" s="4" t="s">
         <v>232</v>
       </c>
       <c r="D16" s="44" t="s">
         <v>106</v>
       </c>
-      <c r="E16" s="54"/>
+      <c r="E16" s="53"/>
       <c r="F16" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="52" t="s">
+      <c r="B17" s="55" t="s">
         <v>132</v>
       </c>
       <c r="C17" s="11" t="s">
@@ -2693,9 +2693,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
-      <c r="B18" s="53"/>
+      <c r="B18" s="56"/>
       <c r="C18" s="4" t="s">
         <v>24</v>
       </c>
@@ -2709,9 +2709,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
-      <c r="B19" s="53"/>
+      <c r="B19" s="56"/>
       <c r="C19" s="11" t="s">
         <v>111</v>
       </c>
@@ -2725,9 +2725,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
-      <c r="B20" s="53"/>
+      <c r="B20" s="56"/>
       <c r="C20" s="11" t="s">
         <v>113</v>
       </c>
@@ -2741,9 +2741,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
-      <c r="B21" s="54"/>
+      <c r="B21" s="53"/>
       <c r="C21" s="11" t="s">
         <v>115</v>
       </c>
@@ -2755,7 +2755,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>133</v>
       </c>
@@ -2773,7 +2773,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" ht="375" x14ac:dyDescent="0.25">
       <c r="A23" s="30" t="s">
         <v>134</v>
       </c>
@@ -2793,7 +2793,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="189" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" ht="210.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>136</v>
       </c>
@@ -2811,11 +2811,11 @@
         <v>140</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="55" t="s">
+    <row r="25" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="57" t="s">
         <v>138</v>
       </c>
-      <c r="B25" s="58" t="s">
+      <c r="B25" s="60" t="s">
         <v>139</v>
       </c>
       <c r="C25" s="9" t="s">
@@ -2831,9 +2831,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="56"/>
-      <c r="B26" s="59"/>
+    <row r="26" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="58"/>
+      <c r="B26" s="61"/>
       <c r="C26" s="9" t="s">
         <v>119</v>
       </c>
@@ -2847,9 +2847,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="56"/>
-      <c r="B27" s="59"/>
+    <row r="27" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="58"/>
+      <c r="B27" s="61"/>
       <c r="C27" s="9" t="s">
         <v>122</v>
       </c>
@@ -2863,9 +2863,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="58" x14ac:dyDescent="0.35">
-      <c r="A28" s="56"/>
-      <c r="B28" s="59"/>
+    <row r="28" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A28" s="58"/>
+      <c r="B28" s="61"/>
       <c r="C28" s="9" t="s">
         <v>125</v>
       </c>
@@ -2879,9 +2879,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="57"/>
-      <c r="B29" s="60"/>
+    <row r="29" spans="1:6" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="59"/>
+      <c r="B29" s="62"/>
       <c r="C29" s="28" t="s">
         <v>128</v>
       </c>
@@ -2889,17 +2889,17 @@
         <v>129</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F29" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B30" s="61" t="s">
+      <c r="B30" s="52" t="s">
         <v>176</v>
       </c>
       <c r="C30" s="3" t="s">
@@ -2908,32 +2908,32 @@
       <c r="D30" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E30" s="62" t="s">
+      <c r="E30" s="54" t="s">
         <v>178</v>
       </c>
       <c r="F30" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="139.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" ht="139.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6"/>
-      <c r="B31" s="54"/>
+      <c r="B31" s="53"/>
       <c r="C31" s="4" t="s">
         <v>233</v>
       </c>
       <c r="D31" s="44" t="s">
         <v>177</v>
       </c>
-      <c r="E31" s="54"/>
+      <c r="E31" s="53"/>
       <c r="F31" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="B32" s="52" t="s">
+      <c r="B32" s="55" t="s">
         <v>179</v>
       </c>
       <c r="C32" s="11" t="s">
@@ -2949,9 +2949,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="6"/>
-      <c r="B33" s="53"/>
+      <c r="B33" s="56"/>
       <c r="C33" s="4" t="s">
         <v>24</v>
       </c>
@@ -2965,9 +2965,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A34" s="6"/>
-      <c r="B34" s="53"/>
+      <c r="B34" s="56"/>
       <c r="C34" s="11" t="s">
         <v>228</v>
       </c>
@@ -2981,9 +2981,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="6"/>
-      <c r="B35" s="53"/>
+      <c r="B35" s="56"/>
       <c r="C35" s="11" t="s">
         <v>181</v>
       </c>
@@ -2997,9 +2997,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="6"/>
-      <c r="B36" s="54"/>
+      <c r="B36" s="53"/>
       <c r="C36" s="11" t="s">
         <v>115</v>
       </c>
@@ -3011,7 +3011,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>187</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" ht="375" x14ac:dyDescent="0.25">
       <c r="A38" s="30" t="s">
         <v>188</v>
       </c>
@@ -3049,29 +3049,29 @@
         <v>175</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="189" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" ht="210.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B39" s="12" t="s">
         <v>242</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>243</v>
       </c>
       <c r="C39" s="12"/>
       <c r="D39" s="51" t="s">
         <v>1</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F39" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="55" t="s">
+    <row r="40" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="57" t="s">
         <v>191</v>
       </c>
-      <c r="B40" s="58" t="s">
+      <c r="B40" s="60" t="s">
         <v>192</v>
       </c>
       <c r="C40" s="9" t="s">
@@ -3087,9 +3087,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="56"/>
-      <c r="B41" s="59"/>
+    <row r="41" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="58"/>
+      <c r="B41" s="61"/>
       <c r="C41" s="9" t="s">
         <v>119</v>
       </c>
@@ -3103,9 +3103,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="56"/>
-      <c r="B42" s="59"/>
+    <row r="42" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="58"/>
+      <c r="B42" s="61"/>
       <c r="C42" s="9" t="s">
         <v>122</v>
       </c>
@@ -3119,9 +3119,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="58" x14ac:dyDescent="0.35">
-      <c r="A43" s="56"/>
-      <c r="B43" s="59"/>
+    <row r="43" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A43" s="58"/>
+      <c r="B43" s="61"/>
       <c r="C43" s="9" t="s">
         <v>193</v>
       </c>
@@ -3135,9 +3135,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="57"/>
-      <c r="B44" s="60"/>
+    <row r="44" spans="1:6" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="59"/>
+      <c r="B44" s="62"/>
       <c r="C44" s="28" t="s">
         <v>194</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>195</v>
       </c>
       <c r="E44" s="28" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F44" t="s">
         <v>175</v>
@@ -3153,11 +3153,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="A40:A44"/>
-    <mergeCell ref="B40:B44"/>
     <mergeCell ref="B17:B21"/>
     <mergeCell ref="A25:A29"/>
     <mergeCell ref="B25:B29"/>
@@ -3166,6 +3161,11 @@
     <mergeCell ref="B4:B8"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="A40:A44"/>
+    <mergeCell ref="B40:B44"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <hyperlinks>
@@ -3213,12 +3213,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C67D23D-5B13-4F00-9F83-043839CEFFD1}">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultColWidth="55.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="55.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="55.453125" style="32"/>
+    <col min="1" max="16384" width="55.42578125" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
         <v>10</v>
       </c>
@@ -3238,11 +3238,11 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="55" t="s">
         <v>61</v>
       </c>
       <c r="C2" s="11" t="s">
@@ -3251,30 +3251,30 @@
       <c r="D2" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="52" t="s">
+      <c r="E2" s="55" t="s">
         <v>66</v>
       </c>
       <c r="F2" s="32" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="30"/>
-      <c r="B3" s="64"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="11" t="s">
         <v>63</v>
       </c>
       <c r="D3" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="64"/>
+      <c r="E3" s="63"/>
       <c r="F3" s="32" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="30"/>
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="55" t="s">
         <v>67</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -3283,32 +3283,32 @@
       <c r="D4" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="52" t="s">
+      <c r="E4" s="55" t="s">
         <v>70</v>
       </c>
       <c r="F4" s="32" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="37"/>
-      <c r="B5" s="63"/>
+      <c r="B5" s="64"/>
       <c r="C5" s="13" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="63"/>
+      <c r="E5" s="64"/>
       <c r="F5" s="32" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="B6" s="52" t="s">
+      <c r="B6" s="55" t="s">
         <v>142</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -3317,30 +3317,30 @@
       <c r="D6" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="E6" s="52" t="s">
+      <c r="E6" s="55" t="s">
         <v>145</v>
       </c>
       <c r="F6" s="32" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="30"/>
-      <c r="B7" s="64"/>
+      <c r="B7" s="63"/>
       <c r="C7" s="11" t="s">
         <v>146</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="E7" s="64"/>
+      <c r="E7" s="63"/>
       <c r="F7" s="32" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="30"/>
-      <c r="B8" s="52" t="s">
+      <c r="B8" s="55" t="s">
         <v>148</v>
       </c>
       <c r="C8" s="11" t="s">
@@ -3349,32 +3349,32 @@
       <c r="D8" s="36" t="s">
         <v>150</v>
       </c>
-      <c r="E8" s="52" t="s">
+      <c r="E8" s="55" t="s">
         <v>151</v>
       </c>
       <c r="F8" s="32" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="37"/>
-      <c r="B9" s="63"/>
+      <c r="B9" s="64"/>
       <c r="C9" s="13" t="s">
         <v>152</v>
       </c>
       <c r="D9" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="E9" s="63"/>
+      <c r="E9" s="64"/>
       <c r="F9" s="32" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="s">
         <v>199</v>
       </c>
-      <c r="B10" s="52" t="s">
+      <c r="B10" s="55" t="s">
         <v>227</v>
       </c>
       <c r="C10" s="11" t="s">
@@ -3383,30 +3383,30 @@
       <c r="D10" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="E10" s="52" t="s">
+      <c r="E10" s="55" t="s">
         <v>205</v>
       </c>
       <c r="F10" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="30"/>
-      <c r="B11" s="64"/>
+      <c r="B11" s="63"/>
       <c r="C11" s="11" t="s">
         <v>202</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="E11" s="64"/>
+      <c r="E11" s="63"/>
       <c r="F11" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="30"/>
-      <c r="B12" s="52" t="s">
+      <c r="B12" s="55" t="s">
         <v>200</v>
       </c>
       <c r="C12" s="11" t="s">
@@ -3415,41 +3415,41 @@
       <c r="D12" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="E12" s="52" t="s">
+      <c r="E12" s="55" t="s">
         <v>206</v>
       </c>
       <c r="F12" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="37"/>
-      <c r="B13" s="63"/>
+      <c r="B13" s="64"/>
       <c r="C13" s="13" t="s">
         <v>204</v>
       </c>
       <c r="D13" s="38" t="s">
         <v>208</v>
       </c>
-      <c r="E13" s="63"/>
+      <c r="E13" s="64"/>
       <c r="F13" s="32" t="s">
         <v>175</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="E6:E7"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="E10:E11"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="E12:E13"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="E8:E9"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="E6:E7"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <hyperlinks>
@@ -3478,9 +3478,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3163888B-9214-4218-82C5-5CD72F2D39D0}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="48.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="48.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -3500,7 +3500,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>25</v>
       </c>
@@ -3518,7 +3518,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>71</v>
       </c>
@@ -3536,7 +3536,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>71</v>
       </c>
@@ -3554,7 +3554,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>153</v>
       </c>
@@ -3572,7 +3572,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>153</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>209</v>
       </c>
@@ -3628,14 +3628,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{172A91E8-EE08-4774-802F-E9F4C78EAB63}">
   <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultColWidth="37.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="37.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="37.26953125" style="32"/>
-    <col min="5" max="5" width="77.26953125" style="32" customWidth="1"/>
-    <col min="6" max="16384" width="37.26953125" style="32"/>
+    <col min="1" max="4" width="37.28515625" style="32"/>
+    <col min="5" max="5" width="77.28515625" style="32" customWidth="1"/>
+    <col min="6" max="16384" width="37.28515625" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
         <v>10</v>
       </c>
@@ -3655,7 +3655,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>74</v>
       </c>
@@ -3675,7 +3675,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="39"/>
       <c r="B3" s="40"/>
       <c r="C3" s="11" t="s">
@@ -3689,7 +3689,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="A4" s="39"/>
       <c r="B4" s="41" t="s">
         <v>100</v>
@@ -3707,7 +3707,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>18</v>
       </c>
@@ -3725,7 +3725,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
         <v>96</v>
       </c>
@@ -3741,7 +3741,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="203" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="255" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
         <v>85</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" ht="240" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
         <v>86</v>
       </c>
@@ -3781,7 +3781,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
         <v>98</v>
       </c>
@@ -3797,7 +3797,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
         <v>99</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
         <v>89</v>
       </c>
@@ -3829,7 +3829,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="25" t="s">
         <v>90</v>
       </c>
@@ -3845,7 +3845,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A13" s="22" t="s">
         <v>156</v>
       </c>
@@ -3865,7 +3865,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="39"/>
       <c r="B14" s="40"/>
       <c r="C14" s="11" t="s">
@@ -3879,7 +3879,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="39"/>
       <c r="B15" s="41" t="s">
         <v>162</v>
@@ -3897,7 +3897,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>18</v>
       </c>
@@ -3915,7 +3915,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="261" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" ht="315" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
         <v>165</v>
       </c>
@@ -3935,7 +3935,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" ht="240" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
         <v>168</v>
       </c>
@@ -3955,7 +3955,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
         <v>98</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="25" t="s">
         <v>99</v>
       </c>
@@ -3991,7 +3991,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A21" s="22" t="s">
         <v>212</v>
       </c>
@@ -4011,7 +4011,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="39"/>
       <c r="B22" s="40"/>
       <c r="C22" s="11" t="s">
@@ -4025,7 +4025,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="174" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" ht="195" x14ac:dyDescent="0.25">
       <c r="A23" s="39"/>
       <c r="B23" s="41" t="s">
         <v>217</v>
@@ -4037,13 +4037,13 @@
         <v>7</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F23" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>18</v>
       </c>
@@ -4061,7 +4061,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="261" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" ht="315" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
         <v>219</v>
       </c>
@@ -4081,7 +4081,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="246.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" ht="300" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
         <v>221</v>
       </c>
@@ -4101,7 +4101,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A27" s="25" t="s">
         <v>98</v>
       </c>
@@ -4119,7 +4119,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
         <v>99</v>
       </c>
@@ -4167,12 +4167,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB73E146-A141-4797-B302-F0B3455C0C2E}">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultColWidth="57.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="57.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="57.54296875" style="32"/>
+    <col min="1" max="16384" width="57.5703125" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
         <v>10</v>
       </c>
@@ -4192,7 +4192,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="31" t="s">
         <v>22</v>
       </c>
@@ -4212,7 +4212,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="31" t="s">
         <v>22</v>
       </c>
@@ -4232,7 +4232,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="31" t="s">
         <v>22</v>
       </c>
@@ -4246,45 +4246,45 @@
         <v>23</v>
       </c>
       <c r="E4" s="49" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="F4" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5" s="16"/>
       <c r="C5" s="17"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B6" s="16"/>
       <c r="C6" s="17"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B7" s="16"/>
       <c r="C7" s="17"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" s="16"/>
       <c r="C8" s="17"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9" s="16"/>
       <c r="C9" s="17"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10" s="16"/>
       <c r="C10" s="17"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11" s="16"/>
       <c r="C11" s="17"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12" s="16"/>
       <c r="C12" s="17"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13" s="16"/>
       <c r="C13" s="17"/>
     </row>
@@ -4299,6 +4299,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="ec07c698-60f5-424f-b9af-f4c59398b511" ContentTypeId="0x010100545E941595ED5448BA61900FDDAFF313" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Official Document" ma:contentTypeID="0x010100545E941595ED5448BA61900FDDAFF31300C0D9F77D091A79449828113EF8250EF5" ma:contentTypeVersion="9" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="3acf8af8f3f036fb6d934619e757bc96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8c566321-f672-4e06-a901-b5e72b4c4357" xmlns:ns3="2a6436df-3f7a-48ac-8ea6-44b411e24bbc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="926947be84ee9a0228ce6a037c6848ba" ns2:_="" ns3:_="">
     <xsd:import namespace="8c566321-f672-4e06-a901-b5e72b4c4357"/>
@@ -4504,12 +4509,61 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="ec07c698-60f5-424f-b9af-f4c59398b511" ContentTypeId="0x010100545E941595ED5448BA61900FDDAFF313" PreviousValue="false"/>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
+      <Value>5</Value>
+      <Value>25</Value>
+      <Value>1</Value>
+      <Value>4</Value>
+    </TaxCatchAll>
+    <p6919dbb65844893b164c5f63a6f0eeb xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">DfE</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">a484111e-5b24-4ad9-9778-c536c8c88985</TermId>
+        </TermInfo>
+      </Terms>
+    </p6919dbb65844893b164c5f63a6f0eeb>
+    <c02f73938b5741d4934b358b31a1b80f xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Official</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">0884c477-2e62-47ea-b19c-5af6e91124c5</TermId>
+        </TermInfo>
+      </Terms>
+    </c02f73938b5741d4934b358b31a1b80f>
+    <f6ec388a6d534bab86a259abd1bfa088 xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">DfE</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">cc08a6d4-dfde-4d0f-bd85-069ebcef80d5</TermId>
+        </TermInfo>
+      </Terms>
+    </f6ec388a6d534bab86a259abd1bfa088>
+    <i98b064926ea4fbe8f5b88c394ff652b xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </i98b064926ea4fbe8f5b88c394ff652b>
+    <_dlc_DocIdUrl xmlns="2a6436df-3f7a-48ac-8ea6-44b411e24bbc">
+      <Url>https://educationgovuk.sharepoint.com/sites/efappp/_layouts/15/DocIdRedir.aspx?ID=FKMV6N5X2MYP-1953928680-76369</Url>
+      <Description>FKMV6N5X2MYP-1953928680-76369</Description>
+    </_dlc_DocIdUrl>
+    <_dlc_DocId xmlns="2a6436df-3f7a-48ac-8ea6-44b411e24bbc">FKMV6N5X2MYP-1953928680-76369</_dlc_DocId>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -4559,61 +4613,15 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D00F0DC4-2D9F-43FC-8616-EC131ED26B7D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
-      <Value>5</Value>
-      <Value>25</Value>
-      <Value>1</Value>
-      <Value>4</Value>
-    </TaxCatchAll>
-    <p6919dbb65844893b164c5f63a6f0eeb xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">DfE</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">a484111e-5b24-4ad9-9778-c536c8c88985</TermId>
-        </TermInfo>
-      </Terms>
-    </p6919dbb65844893b164c5f63a6f0eeb>
-    <c02f73938b5741d4934b358b31a1b80f xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Official</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">0884c477-2e62-47ea-b19c-5af6e91124c5</TermId>
-        </TermInfo>
-      </Terms>
-    </c02f73938b5741d4934b358b31a1b80f>
-    <f6ec388a6d534bab86a259abd1bfa088 xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">DfE</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">cc08a6d4-dfde-4d0f-bd85-069ebcef80d5</TermId>
-        </TermInfo>
-      </Terms>
-    </f6ec388a6d534bab86a259abd1bfa088>
-    <i98b064926ea4fbe8f5b88c394ff652b xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </i98b064926ea4fbe8f5b88c394ff652b>
-    <_dlc_DocIdUrl xmlns="2a6436df-3f7a-48ac-8ea6-44b411e24bbc">
-      <Url>https://educationgovuk.sharepoint.com/sites/efappp/_layouts/15/DocIdRedir.aspx?ID=FKMV6N5X2MYP-1953928680-76369</Url>
-      <Description>FKMV6N5X2MYP-1953928680-76369</Description>
-    </_dlc_DocIdUrl>
-    <_dlc_DocId xmlns="2a6436df-3f7a-48ac-8ea6-44b411e24bbc">FKMV6N5X2MYP-1953928680-76369</_dlc_DocId>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1E94FF3-D2F7-4169-BE5C-5ED202BAA024}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4632,31 +4640,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D00F0DC4-2D9F-43FC-8616-EC131ED26B7D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9C56A4F-6917-41AA-BBE5-DA7C75896563}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035EEA42-582A-4724-B162-C22729062C2B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{334E8BC2-6B82-4EDA-BE50-EFE4767E8CD2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="8c566321-f672-4e06-a901-b5e72b4c4357"/>
@@ -4673,6 +4657,22 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035EEA42-582A-4724-B162-C22729062C2B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9C56A4F-6917-41AA-BBE5-DA7C75896563}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{de278828-447b-4aaa-a336-d38da9839a3c}" enabled="1" method="Privileged" siteId="{fad277c9-c60a-4da1-b5f3-b3b8b34a82f9}" contentBits="3" removed="0"/>

</xml_diff>

<commit_message>
changes to forecast accuracy chart and technical guidance (#130)
</commit_message>
<xml_diff>
--- a/data/tech_guidance.xlsx
+++ b/data/tech_guidance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rmiller3\repos\la-school-places-scorecard-internal\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jbrett\repos\la-school-places-scorecards\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62591664-EEA0-428C-BFDE-3207C90A1360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12CB439D-05BA-4DB1-B6A5-55831A0081A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{9CCC1F63-2262-45DD-B4CA-7C937E5C8E7F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{9CCC1F63-2262-45DD-B4CA-7C937E5C8E7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Quantity" sheetId="2" r:id="rId1"/>
@@ -1361,6 +1361,39 @@
     </r>
   </si>
   <si>
+    <t>1. Each school has been matched with the Ofsted data as at  31 August 2025 (published November 2025). Graded judgements on four areas 'Quality of Education', 'Behaviour and Attitudes', 'Personal Development' and 'Leadership and Management' are used and where the inspection took place before 1 September 2023 the rating for 'Overall effectiveness: how good is the school is." is used for each judgement area.
+&lt;br&gt;2. There are four Ofsted categories: 'Outstanding', 'Good', 'Requires improvement' and 'Inadequate'.
+&lt;br&gt;3. The calculation counts the number of existing and new places that have been created in schools of each category. &lt;br&gt;4. Note that many schools will have been inspected some time before August 2025, and some will have been inspected since this date. &lt;br&gt;5. There are school places with no rating, as the school has yet to be inspected so do not have an Ofsted judgement.</t>
+  </si>
+  <si>
+    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2027/28 as provided in SCAP 2025.
+&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
+&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
+&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
+  </si>
+  <si>
+    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2026/27 as provided in SCAP 2024.
+&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
+&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
+&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
+  </si>
+  <si>
+    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2025/26 as provided in SCAP 2023.
+&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
+&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
+&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
+  </si>
+  <si>
+    <t>Total basic need funding 2011 to 2028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total amount of basic need capital funding allocated to each local authority to support them to create new mainstream primary and secondary places from 2011 to 2028. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. This refers to the amount of basic need capital funding that the Department for Education (DfE) has allocated to each local authority to create new places from the 2011-12 financial year to the 2027-28 financial year. Basic Need funding for the 2027-28 financial year is intended to support the creation of mainstream places for pupils aged 5 to 16 for the 2028/29 academic year. &lt;br&gt;2. The figure includes formula-based funding allocations and funding provided through the Targeted Basic Need Programme. Basic Need formula-based funding allocations cover the whole period and are not ring-fenced (although they can only be used for capital purposes).  Targeted Basic Need funding was provided between 2013 and 2015 and had to be spent by agreed deadlines and on specific projects. Both types of allocations are published here. &lt;br&gt;3. The figure only includes funding allocated to local authorities and does not include centrally-funded capital programmes such as the free schools programme. &lt;br&gt;4. The England total will not match the sum of allocations for all local authorities in the scorecard because the England total includes allocations to predecessor local authorities.
+</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">1. The cost data used in the scorecard is the 2018 Capital Spend data as used in the scorecards since 2018. For the 2025 Scorecard, this data has been adjusted for inflation (rebased to 1st Quarter 2026 prices). National averages adjusted for 2023 regional location factors are shown. You can use this data to establish developer contributions per school place, by adjusting for further inflation if needed (see examples below).
 &lt;br&gt;2. Projects which do not create additional mainstream places or where the project's additional place funding is zero are removed.
@@ -1465,7 +1498,7 @@
 &lt;br&gt;6. The average cost includes costs associated with maintenance and building condition or enhancement works.
 &lt;br&gt;7. The measure does not include places in special schools or units attached to mainstream schools, or new places which were funded through central programmes (including free schools). For projects within the 2018 Capital Spend dataset, a project which creates additional mainstream places and also creates SEN places or re-provides places, has been adjusted to apportion out those costs. For projects within the Capital Spend Survey, apportioning costs is not possible and therefore a project which creates additional mainstream places and also creates SEN places or re-provides places has been excluded.
 &lt;br&gt;8. All costs have been normalised to a common UK average price level using regional location factors published by BCIS, March 2023, 1 is the base weight.
-&lt;br&gt;9. All costs have been adjusted for inflation using the latest BCIS All-In Tender Price of Index (TPI), published March 2026.  Costs have been rebased from the start of construction (or time of place provision if construction start date unavailable) to 1st Quarter (Jan – Mar) 2026 prices using this index (Q1 2026 index value = 399).
+&lt;br&gt;9. All costs have been adjusted for inflation using the latest BCIS All-In Tender Price of Index (TPI), published March 2026.  Costs have been rebased from the start of construction (or time of place provision if construction start date unavailable) to 1st Quarter (Jan – Mar) 2026 prices using this index (Q1 2026 index value = 410).
 10. </t>
     </r>
     <r>
@@ -1485,42 +1518,9 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>.  If you have access to the BCIS indices via a subscription to BCIS Online (https://www.rics.org/uk/products/data-products/bcis-construction/bcis-online/) you can use the latest inflation index to re-base (weight to apply = latest index/399).  If not, you can apply a known change to the published cost (e.g. up or down x%).
+      <t>.  If you have access to the BCIS indices via a subscription to BCIS Online (https://www.rics.org/uk/products/data-products/bcis-construction/bcis-online/) you can use the latest inflation index to re-base (weight to apply = latest index/410).  If not, you can apply a known change to the published cost (e.g. up or down x%).
 11. Some additional but limited benchmark information for similar capital programme schemes carried out by the DfE is available in the National School Delivery Cost Benchmarking study: https://documents.hants.gov.uk/property-services/NationalSchoolDeliveryBenchmarkingreport.pdf</t>
     </r>
-  </si>
-  <si>
-    <t>1. Each school has been matched with the Ofsted data as at  31 August 2025 (published November 2025). Graded judgements on four areas 'Quality of Education', 'Behaviour and Attitudes', 'Personal Development' and 'Leadership and Management' are used and where the inspection took place before 1 September 2023 the rating for 'Overall effectiveness: how good is the school is." is used for each judgement area.
-&lt;br&gt;2. There are four Ofsted categories: 'Outstanding', 'Good', 'Requires improvement' and 'Inadequate'.
-&lt;br&gt;3. The calculation counts the number of existing and new places that have been created in schools of each category. &lt;br&gt;4. Note that many schools will have been inspected some time before August 2025, and some will have been inspected since this date. &lt;br&gt;5. There are school places with no rating, as the school has yet to be inspected so do not have an Ofsted judgement.</t>
-  </si>
-  <si>
-    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2027/28 as provided in SCAP 2025.
-&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
-&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
-&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
-  </si>
-  <si>
-    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2026/27 as provided in SCAP 2024.
-&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
-&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
-&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
-  </si>
-  <si>
-    <t>1. This is the local authority's forecast of pupil numbers for the academic year 2025/26 as provided in SCAP 2023.
-&lt;br&gt;2. These forecasts cover pupils that local authorities anticipate will attend primary schools (or primary provision in middle or all-through schools i.e. years R-6) and secondary schools (or secondary provision in middle or all-through schools i.e. years 7-11)
-&lt;br&gt;3. These forecasts focus on local authorities expectations about new school places and do not include pupils who are expected to attend independent schools or special/non-mainstream provision.
-&lt;br&gt;4. Anticipated change in pupil numbers should be viewed in conjunction with an LAs forecast accuracy. Low one-year out forecast accuracy may result in the anticipated change in pupil numbers not being representative of the trend of an LAs pupil number forecasts.</t>
-  </si>
-  <si>
-    <t>Total basic need funding 2011 to 2028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total amount of basic need capital funding allocated to each local authority to support them to create new mainstream primary and secondary places from 2011 to 2028. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. This refers to the amount of basic need capital funding that the Department for Education (DfE) has allocated to each local authority to create new places from the 2011-12 financial year to the 2027-28 financial year. Basic Need funding for the 2027-28 financial year is intended to support the creation of mainstream places for pupils aged 5 to 16 for the 2028/29 academic year. &lt;br&gt;2. The figure includes formula-based funding allocations and funding provided through the Targeted Basic Need Programme. Basic Need formula-based funding allocations cover the whole period and are not ring-fenced (although they can only be used for capital purposes).  Targeted Basic Need funding was provided between 2013 and 2015 and had to be spent by agreed deadlines and on specific projects. Both types of allocations are published here. &lt;br&gt;3. The figure only includes funding allocated to local authorities and does not include centrally-funded capital programmes such as the free schools programme. &lt;br&gt;4. The England total will not match the sum of allocations for all local authorities in the scorecard because the England total includes allocations to predecessor local authorities.
-</t>
   </si>
 </sst>
 </file>
@@ -2031,15 +2031,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2058,16 +2064,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2386,16 +2386,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8372DA64-5E2C-41C1-8CF4-85BC1C2AFF86}">
   <dimension ref="A1:F44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.7265625" customWidth="1"/>
-    <col min="2" max="2" width="29.54296875" customWidth="1"/>
-    <col min="3" max="3" width="54.26953125" customWidth="1"/>
-    <col min="4" max="4" width="28.7265625" customWidth="1"/>
-    <col min="5" max="5" width="87.26953125" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.5703125" customWidth="1"/>
+    <col min="3" max="3" width="54.28515625" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" customWidth="1"/>
+    <col min="5" max="5" width="87.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -2415,11 +2415,11 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="87" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="52" t="s">
         <v>33</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -2428,32 +2428,32 @@
       <c r="D2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="62" t="s">
+      <c r="E2" s="54" t="s">
         <v>34</v>
       </c>
       <c r="F2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="87" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
-      <c r="B3" s="54"/>
+      <c r="B3" s="53"/>
       <c r="C3" s="4" t="s">
         <v>231</v>
       </c>
       <c r="D3" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="54"/>
+      <c r="E3" s="53"/>
       <c r="F3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="138" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="138" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="55" t="s">
         <v>94</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -2469,9 +2469,9 @@
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
-      <c r="B5" s="53"/>
+      <c r="B5" s="56"/>
       <c r="C5" s="4" t="s">
         <v>24</v>
       </c>
@@ -2485,9 +2485,9 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
-      <c r="B6" s="53"/>
+      <c r="B6" s="56"/>
       <c r="C6" s="11" t="s">
         <v>42</v>
       </c>
@@ -2501,9 +2501,9 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="6"/>
-      <c r="B7" s="53"/>
+      <c r="B7" s="56"/>
       <c r="C7" s="11" t="s">
         <v>43</v>
       </c>
@@ -2517,9 +2517,9 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
-      <c r="B8" s="54"/>
+      <c r="B8" s="53"/>
       <c r="C8" s="11" t="s">
         <v>229</v>
       </c>
@@ -2531,7 +2531,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>46</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="375" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="s">
         <v>47</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="189" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" ht="210.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>50</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
         <v>54</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
       <c r="B13" s="19"/>
       <c r="C13" s="9" t="s">
@@ -2623,7 +2623,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7"/>
       <c r="B14" s="24"/>
       <c r="C14" s="28" t="s">
@@ -2633,17 +2633,17 @@
         <v>59</v>
       </c>
       <c r="E14" s="28" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F14" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="61" t="s">
+      <c r="B15" s="52" t="s">
         <v>130</v>
       </c>
       <c r="C15" s="3" t="s">
@@ -2652,32 +2652,32 @@
       <c r="D15" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E15" s="62" t="s">
+      <c r="E15" s="54" t="s">
         <v>105</v>
       </c>
       <c r="F15" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
-      <c r="B16" s="54"/>
+      <c r="B16" s="53"/>
       <c r="C16" s="4" t="s">
         <v>232</v>
       </c>
       <c r="D16" s="44" t="s">
         <v>106</v>
       </c>
-      <c r="E16" s="54"/>
+      <c r="E16" s="53"/>
       <c r="F16" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="52" t="s">
+      <c r="B17" s="55" t="s">
         <v>132</v>
       </c>
       <c r="C17" s="11" t="s">
@@ -2693,9 +2693,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
-      <c r="B18" s="53"/>
+      <c r="B18" s="56"/>
       <c r="C18" s="4" t="s">
         <v>24</v>
       </c>
@@ -2709,9 +2709,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
-      <c r="B19" s="53"/>
+      <c r="B19" s="56"/>
       <c r="C19" s="11" t="s">
         <v>111</v>
       </c>
@@ -2725,9 +2725,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
-      <c r="B20" s="53"/>
+      <c r="B20" s="56"/>
       <c r="C20" s="11" t="s">
         <v>113</v>
       </c>
@@ -2741,9 +2741,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
-      <c r="B21" s="54"/>
+      <c r="B21" s="53"/>
       <c r="C21" s="11" t="s">
         <v>115</v>
       </c>
@@ -2755,7 +2755,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>133</v>
       </c>
@@ -2773,7 +2773,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" ht="375" x14ac:dyDescent="0.25">
       <c r="A23" s="30" t="s">
         <v>134</v>
       </c>
@@ -2793,7 +2793,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="189" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" ht="210.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>136</v>
       </c>
@@ -2811,11 +2811,11 @@
         <v>140</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="55" t="s">
+    <row r="25" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="57" t="s">
         <v>138</v>
       </c>
-      <c r="B25" s="58" t="s">
+      <c r="B25" s="60" t="s">
         <v>139</v>
       </c>
       <c r="C25" s="9" t="s">
@@ -2831,9 +2831,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="56"/>
-      <c r="B26" s="59"/>
+    <row r="26" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="58"/>
+      <c r="B26" s="61"/>
       <c r="C26" s="9" t="s">
         <v>119</v>
       </c>
@@ -2847,9 +2847,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="56"/>
-      <c r="B27" s="59"/>
+    <row r="27" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="58"/>
+      <c r="B27" s="61"/>
       <c r="C27" s="9" t="s">
         <v>122</v>
       </c>
@@ -2863,9 +2863,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="58" x14ac:dyDescent="0.35">
-      <c r="A28" s="56"/>
-      <c r="B28" s="59"/>
+    <row r="28" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A28" s="58"/>
+      <c r="B28" s="61"/>
       <c r="C28" s="9" t="s">
         <v>125</v>
       </c>
@@ -2879,9 +2879,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="57"/>
-      <c r="B29" s="60"/>
+    <row r="29" spans="1:6" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="59"/>
+      <c r="B29" s="62"/>
       <c r="C29" s="28" t="s">
         <v>128</v>
       </c>
@@ -2889,17 +2889,17 @@
         <v>129</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F29" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B30" s="61" t="s">
+      <c r="B30" s="52" t="s">
         <v>176</v>
       </c>
       <c r="C30" s="3" t="s">
@@ -2908,32 +2908,32 @@
       <c r="D30" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E30" s="62" t="s">
+      <c r="E30" s="54" t="s">
         <v>178</v>
       </c>
       <c r="F30" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="139.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" ht="139.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6"/>
-      <c r="B31" s="54"/>
+      <c r="B31" s="53"/>
       <c r="C31" s="4" t="s">
         <v>233</v>
       </c>
       <c r="D31" s="44" t="s">
         <v>177</v>
       </c>
-      <c r="E31" s="54"/>
+      <c r="E31" s="53"/>
       <c r="F31" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="B32" s="52" t="s">
+      <c r="B32" s="55" t="s">
         <v>179</v>
       </c>
       <c r="C32" s="11" t="s">
@@ -2949,9 +2949,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="6"/>
-      <c r="B33" s="53"/>
+      <c r="B33" s="56"/>
       <c r="C33" s="4" t="s">
         <v>24</v>
       </c>
@@ -2965,9 +2965,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A34" s="6"/>
-      <c r="B34" s="53"/>
+      <c r="B34" s="56"/>
       <c r="C34" s="11" t="s">
         <v>228</v>
       </c>
@@ -2981,9 +2981,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="6"/>
-      <c r="B35" s="53"/>
+      <c r="B35" s="56"/>
       <c r="C35" s="11" t="s">
         <v>181</v>
       </c>
@@ -2997,9 +2997,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="6"/>
-      <c r="B36" s="54"/>
+      <c r="B36" s="53"/>
       <c r="C36" s="11" t="s">
         <v>115</v>
       </c>
@@ -3011,7 +3011,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>187</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" ht="375" x14ac:dyDescent="0.25">
       <c r="A38" s="30" t="s">
         <v>188</v>
       </c>
@@ -3049,29 +3049,29 @@
         <v>175</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="189" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" ht="210.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B39" s="12" t="s">
         <v>242</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>243</v>
       </c>
       <c r="C39" s="12"/>
       <c r="D39" s="51" t="s">
         <v>1</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F39" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="55" t="s">
+    <row r="40" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="57" t="s">
         <v>191</v>
       </c>
-      <c r="B40" s="58" t="s">
+      <c r="B40" s="60" t="s">
         <v>192</v>
       </c>
       <c r="C40" s="9" t="s">
@@ -3087,9 +3087,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="56"/>
-      <c r="B41" s="59"/>
+    <row r="41" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="58"/>
+      <c r="B41" s="61"/>
       <c r="C41" s="9" t="s">
         <v>119</v>
       </c>
@@ -3103,9 +3103,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="56"/>
-      <c r="B42" s="59"/>
+    <row r="42" spans="1:6" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="58"/>
+      <c r="B42" s="61"/>
       <c r="C42" s="9" t="s">
         <v>122</v>
       </c>
@@ -3119,9 +3119,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="58" x14ac:dyDescent="0.35">
-      <c r="A43" s="56"/>
-      <c r="B43" s="59"/>
+    <row r="43" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A43" s="58"/>
+      <c r="B43" s="61"/>
       <c r="C43" s="9" t="s">
         <v>193</v>
       </c>
@@ -3135,9 +3135,9 @@
         <v>175</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="57"/>
-      <c r="B44" s="60"/>
+    <row r="44" spans="1:6" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="59"/>
+      <c r="B44" s="62"/>
       <c r="C44" s="28" t="s">
         <v>194</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>195</v>
       </c>
       <c r="E44" s="28" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F44" t="s">
         <v>175</v>
@@ -3153,11 +3153,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="B32:B36"/>
-    <mergeCell ref="A40:A44"/>
-    <mergeCell ref="B40:B44"/>
     <mergeCell ref="B17:B21"/>
     <mergeCell ref="A25:A29"/>
     <mergeCell ref="B25:B29"/>
@@ -3166,6 +3161,11 @@
     <mergeCell ref="B4:B8"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="B32:B36"/>
+    <mergeCell ref="A40:A44"/>
+    <mergeCell ref="B40:B44"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <hyperlinks>
@@ -3213,12 +3213,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C67D23D-5B13-4F00-9F83-043839CEFFD1}">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultColWidth="55.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="55.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="55.453125" style="32"/>
+    <col min="1" max="16384" width="55.42578125" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
         <v>10</v>
       </c>
@@ -3238,11 +3238,11 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="55" t="s">
         <v>61</v>
       </c>
       <c r="C2" s="11" t="s">
@@ -3251,30 +3251,30 @@
       <c r="D2" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="52" t="s">
+      <c r="E2" s="55" t="s">
         <v>66</v>
       </c>
       <c r="F2" s="32" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="30"/>
-      <c r="B3" s="64"/>
+      <c r="B3" s="63"/>
       <c r="C3" s="11" t="s">
         <v>63</v>
       </c>
       <c r="D3" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="64"/>
+      <c r="E3" s="63"/>
       <c r="F3" s="32" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="30"/>
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="55" t="s">
         <v>67</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -3283,32 +3283,32 @@
       <c r="D4" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="52" t="s">
+      <c r="E4" s="55" t="s">
         <v>70</v>
       </c>
       <c r="F4" s="32" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="37"/>
-      <c r="B5" s="63"/>
+      <c r="B5" s="64"/>
       <c r="C5" s="13" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="63"/>
+      <c r="E5" s="64"/>
       <c r="F5" s="32" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="B6" s="52" t="s">
+      <c r="B6" s="55" t="s">
         <v>142</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -3317,30 +3317,30 @@
       <c r="D6" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="E6" s="52" t="s">
+      <c r="E6" s="55" t="s">
         <v>145</v>
       </c>
       <c r="F6" s="32" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="30"/>
-      <c r="B7" s="64"/>
+      <c r="B7" s="63"/>
       <c r="C7" s="11" t="s">
         <v>146</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="E7" s="64"/>
+      <c r="E7" s="63"/>
       <c r="F7" s="32" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="30"/>
-      <c r="B8" s="52" t="s">
+      <c r="B8" s="55" t="s">
         <v>148</v>
       </c>
       <c r="C8" s="11" t="s">
@@ -3349,32 +3349,32 @@
       <c r="D8" s="36" t="s">
         <v>150</v>
       </c>
-      <c r="E8" s="52" t="s">
+      <c r="E8" s="55" t="s">
         <v>151</v>
       </c>
       <c r="F8" s="32" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="37"/>
-      <c r="B9" s="63"/>
+      <c r="B9" s="64"/>
       <c r="C9" s="13" t="s">
         <v>152</v>
       </c>
       <c r="D9" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="E9" s="63"/>
+      <c r="E9" s="64"/>
       <c r="F9" s="32" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="s">
         <v>199</v>
       </c>
-      <c r="B10" s="52" t="s">
+      <c r="B10" s="55" t="s">
         <v>227</v>
       </c>
       <c r="C10" s="11" t="s">
@@ -3383,30 +3383,30 @@
       <c r="D10" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="E10" s="52" t="s">
+      <c r="E10" s="55" t="s">
         <v>205</v>
       </c>
       <c r="F10" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="30"/>
-      <c r="B11" s="64"/>
+      <c r="B11" s="63"/>
       <c r="C11" s="11" t="s">
         <v>202</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="E11" s="64"/>
+      <c r="E11" s="63"/>
       <c r="F11" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="30"/>
-      <c r="B12" s="52" t="s">
+      <c r="B12" s="55" t="s">
         <v>200</v>
       </c>
       <c r="C12" s="11" t="s">
@@ -3415,41 +3415,41 @@
       <c r="D12" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="E12" s="52" t="s">
+      <c r="E12" s="55" t="s">
         <v>206</v>
       </c>
       <c r="F12" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="37"/>
-      <c r="B13" s="63"/>
+      <c r="B13" s="64"/>
       <c r="C13" s="13" t="s">
         <v>204</v>
       </c>
       <c r="D13" s="38" t="s">
         <v>208</v>
       </c>
-      <c r="E13" s="63"/>
+      <c r="E13" s="64"/>
       <c r="F13" s="32" t="s">
         <v>175</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="E6:E7"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="E10:E11"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="E12:E13"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="E8:E9"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="E6:E7"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <hyperlinks>
@@ -3478,9 +3478,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3163888B-9214-4218-82C5-5CD72F2D39D0}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="48.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="48.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -3500,7 +3500,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>25</v>
       </c>
@@ -3518,7 +3518,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>71</v>
       </c>
@@ -3536,7 +3536,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>71</v>
       </c>
@@ -3554,7 +3554,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>153</v>
       </c>
@@ -3572,7 +3572,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>153</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>209</v>
       </c>
@@ -3628,14 +3628,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{172A91E8-EE08-4774-802F-E9F4C78EAB63}">
   <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultColWidth="37.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="37.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="37.26953125" style="32"/>
-    <col min="5" max="5" width="77.26953125" style="32" customWidth="1"/>
-    <col min="6" max="16384" width="37.26953125" style="32"/>
+    <col min="1" max="4" width="37.28515625" style="32"/>
+    <col min="5" max="5" width="77.28515625" style="32" customWidth="1"/>
+    <col min="6" max="16384" width="37.28515625" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
         <v>10</v>
       </c>
@@ -3655,7 +3655,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>74</v>
       </c>
@@ -3675,7 +3675,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="39"/>
       <c r="B3" s="40"/>
       <c r="C3" s="11" t="s">
@@ -3689,7 +3689,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="A4" s="39"/>
       <c r="B4" s="41" t="s">
         <v>100</v>
@@ -3707,7 +3707,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>18</v>
       </c>
@@ -3725,7 +3725,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
         <v>96</v>
       </c>
@@ -3741,7 +3741,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="203" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="255" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
         <v>85</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" ht="240" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
         <v>86</v>
       </c>
@@ -3781,7 +3781,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
         <v>98</v>
       </c>
@@ -3797,7 +3797,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
         <v>99</v>
       </c>
@@ -3813,7 +3813,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
         <v>89</v>
       </c>
@@ -3829,7 +3829,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="25" t="s">
         <v>90</v>
       </c>
@@ -3845,7 +3845,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A13" s="22" t="s">
         <v>156</v>
       </c>
@@ -3865,7 +3865,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="39"/>
       <c r="B14" s="40"/>
       <c r="C14" s="11" t="s">
@@ -3879,7 +3879,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="39"/>
       <c r="B15" s="41" t="s">
         <v>162</v>
@@ -3897,7 +3897,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>18</v>
       </c>
@@ -3915,7 +3915,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="261" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" ht="315" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
         <v>165</v>
       </c>
@@ -3935,7 +3935,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" ht="240" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
         <v>168</v>
       </c>
@@ -3955,7 +3955,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
         <v>98</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="25" t="s">
         <v>99</v>
       </c>
@@ -3991,7 +3991,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A21" s="22" t="s">
         <v>212</v>
       </c>
@@ -4011,7 +4011,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="39"/>
       <c r="B22" s="40"/>
       <c r="C22" s="11" t="s">
@@ -4025,7 +4025,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="174" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" ht="195" x14ac:dyDescent="0.25">
       <c r="A23" s="39"/>
       <c r="B23" s="41" t="s">
         <v>217</v>
@@ -4037,13 +4037,13 @@
         <v>7</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F23" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>18</v>
       </c>
@@ -4061,7 +4061,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="261" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" ht="315" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
         <v>219</v>
       </c>
@@ -4081,7 +4081,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="246.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" ht="300" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
         <v>221</v>
       </c>
@@ -4101,7 +4101,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A27" s="25" t="s">
         <v>98</v>
       </c>
@@ -4119,7 +4119,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
         <v>99</v>
       </c>
@@ -4167,12 +4167,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB73E146-A141-4797-B302-F0B3455C0C2E}">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultColWidth="57.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="57.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="57.54296875" style="32"/>
+    <col min="1" max="16384" width="57.5703125" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
         <v>10</v>
       </c>
@@ -4192,7 +4192,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="31" t="s">
         <v>22</v>
       </c>
@@ -4212,7 +4212,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="31" t="s">
         <v>22</v>
       </c>
@@ -4232,7 +4232,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="31" t="s">
         <v>22</v>
       </c>
@@ -4246,45 +4246,45 @@
         <v>23</v>
       </c>
       <c r="E4" s="49" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="F4" s="32" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5" s="16"/>
       <c r="C5" s="17"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B6" s="16"/>
       <c r="C6" s="17"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B7" s="16"/>
       <c r="C7" s="17"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" s="16"/>
       <c r="C8" s="17"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9" s="16"/>
       <c r="C9" s="17"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10" s="16"/>
       <c r="C10" s="17"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11" s="16"/>
       <c r="C11" s="17"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12" s="16"/>
       <c r="C12" s="17"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13" s="16"/>
       <c r="C13" s="17"/>
     </row>
@@ -4299,6 +4299,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="ec07c698-60f5-424f-b9af-f4c59398b511" ContentTypeId="0x010100545E941595ED5448BA61900FDDAFF313" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Official Document" ma:contentTypeID="0x010100545E941595ED5448BA61900FDDAFF31300C0D9F77D091A79449828113EF8250EF5" ma:contentTypeVersion="9" ma:contentTypeDescription="" ma:contentTypeScope="" ma:versionID="3acf8af8f3f036fb6d934619e757bc96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8c566321-f672-4e06-a901-b5e72b4c4357" xmlns:ns3="2a6436df-3f7a-48ac-8ea6-44b411e24bbc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="926947be84ee9a0228ce6a037c6848ba" ns2:_="" ns3:_="">
     <xsd:import namespace="8c566321-f672-4e06-a901-b5e72b4c4357"/>
@@ -4504,12 +4509,61 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="ec07c698-60f5-424f-b9af-f4c59398b511" ContentTypeId="0x010100545E941595ED5448BA61900FDDAFF313" PreviousValue="false"/>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
+      <Value>5</Value>
+      <Value>25</Value>
+      <Value>1</Value>
+      <Value>4</Value>
+    </TaxCatchAll>
+    <p6919dbb65844893b164c5f63a6f0eeb xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">DfE</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">a484111e-5b24-4ad9-9778-c536c8c88985</TermId>
+        </TermInfo>
+      </Terms>
+    </p6919dbb65844893b164c5f63a6f0eeb>
+    <c02f73938b5741d4934b358b31a1b80f xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Official</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">0884c477-2e62-47ea-b19c-5af6e91124c5</TermId>
+        </TermInfo>
+      </Terms>
+    </c02f73938b5741d4934b358b31a1b80f>
+    <f6ec388a6d534bab86a259abd1bfa088 xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">DfE</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">cc08a6d4-dfde-4d0f-bd85-069ebcef80d5</TermId>
+        </TermInfo>
+      </Terms>
+    </f6ec388a6d534bab86a259abd1bfa088>
+    <i98b064926ea4fbe8f5b88c394ff652b xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </i98b064926ea4fbe8f5b88c394ff652b>
+    <_dlc_DocIdUrl xmlns="2a6436df-3f7a-48ac-8ea6-44b411e24bbc">
+      <Url>https://educationgovuk.sharepoint.com/sites/efappp/_layouts/15/DocIdRedir.aspx?ID=FKMV6N5X2MYP-1953928680-76369</Url>
+      <Description>FKMV6N5X2MYP-1953928680-76369</Description>
+    </_dlc_DocIdUrl>
+    <_dlc_DocId xmlns="2a6436df-3f7a-48ac-8ea6-44b411e24bbc">FKMV6N5X2MYP-1953928680-76369</_dlc_DocId>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -4559,61 +4613,15 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D00F0DC4-2D9F-43FC-8616-EC131ED26B7D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
-      <Value>5</Value>
-      <Value>25</Value>
-      <Value>1</Value>
-      <Value>4</Value>
-    </TaxCatchAll>
-    <p6919dbb65844893b164c5f63a6f0eeb xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">DfE</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">a484111e-5b24-4ad9-9778-c536c8c88985</TermId>
-        </TermInfo>
-      </Terms>
-    </p6919dbb65844893b164c5f63a6f0eeb>
-    <c02f73938b5741d4934b358b31a1b80f xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Official</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">0884c477-2e62-47ea-b19c-5af6e91124c5</TermId>
-        </TermInfo>
-      </Terms>
-    </c02f73938b5741d4934b358b31a1b80f>
-    <f6ec388a6d534bab86a259abd1bfa088 xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">DfE</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">cc08a6d4-dfde-4d0f-bd85-069ebcef80d5</TermId>
-        </TermInfo>
-      </Terms>
-    </f6ec388a6d534bab86a259abd1bfa088>
-    <i98b064926ea4fbe8f5b88c394ff652b xmlns="8c566321-f672-4e06-a901-b5e72b4c4357">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </i98b064926ea4fbe8f5b88c394ff652b>
-    <_dlc_DocIdUrl xmlns="2a6436df-3f7a-48ac-8ea6-44b411e24bbc">
-      <Url>https://educationgovuk.sharepoint.com/sites/efappp/_layouts/15/DocIdRedir.aspx?ID=FKMV6N5X2MYP-1953928680-76369</Url>
-      <Description>FKMV6N5X2MYP-1953928680-76369</Description>
-    </_dlc_DocIdUrl>
-    <_dlc_DocId xmlns="2a6436df-3f7a-48ac-8ea6-44b411e24bbc">FKMV6N5X2MYP-1953928680-76369</_dlc_DocId>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F1E94FF3-D2F7-4169-BE5C-5ED202BAA024}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4632,31 +4640,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D00F0DC4-2D9F-43FC-8616-EC131ED26B7D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9C56A4F-6917-41AA-BBE5-DA7C75896563}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035EEA42-582A-4724-B162-C22729062C2B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{334E8BC2-6B82-4EDA-BE50-EFE4767E8CD2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="8c566321-f672-4e06-a901-b5e72b4c4357"/>
@@ -4673,6 +4657,22 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035EEA42-582A-4724-B162-C22729062C2B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9C56A4F-6917-41AA-BBE5-DA7C75896563}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{de278828-447b-4aaa-a336-d38da9839a3c}" enabled="1" method="Privileged" siteId="{fad277c9-c60a-4da1-b5f3-b3b8b34a82f9}" contentBits="3" removed="0"/>

</xml_diff>